<commit_message>
08-06-2026 Updated After S3 Bucket
</commit_message>
<xml_diff>
--- a/Wikidata Delta/om_gen_excels/pep_oman_living_relevant_cleaned.xlsx
+++ b/Wikidata Delta/om_gen_excels/pep_oman_living_relevant_cleaned.xlsx
@@ -715,7 +715,7 @@
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V2" t="n">
@@ -746,12 +746,12 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE2" t="inlineStr">
         <is>
-          <t>['Shakoor Bint Mohammed Al Ghammari', 'Shakour Bint Mohammed Al Ghamari']</t>
+          <t>['Shakour Bint Mohammed Al Ghamari', 'শকুর বিনতে মোহাম্মদ আল ঘামারি', 'شکور بنت محمد الغماری', 'Shakoor Bint Mohammed Al Ghammari']</t>
         </is>
       </c>
       <c r="AF2" t="inlineStr">
@@ -885,7 +885,7 @@
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V3" t="n">
@@ -916,12 +916,12 @@
       </c>
       <c r="AD3" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE3" t="inlineStr">
         <is>
-          <t>['Taiba Al Mawali']</t>
+          <t>['তাইবা আল মাওয়ালি', 'طیبہ الموالی', 'Taiba Al Mawali']</t>
         </is>
       </c>
       <c r="AF3" t="inlineStr">
@@ -1059,7 +1059,7 @@
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V4" t="n">
@@ -1090,12 +1090,12 @@
       </c>
       <c r="AD4" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>['Lujaina Mohsin Haider Darwish', 'Lujaina Mohsin Darwish']</t>
+          <t>['লুজাইনা মহসিন দারভিশ', 'Lujaina Mohsin Haider Darwish', 'Lujaina Mohsin Darwish', 'لجينة محسن درويش', 'لجینہ محسن درویش']</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -1233,7 +1233,7 @@
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V5" t="n">
@@ -1264,12 +1264,12 @@
       </c>
       <c r="AD5" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>['Areej Darwish', 'Areej Mohsin Darwish', 'Areej Mohsin Haider Darwish Al Zaabi', 'Areej Mohsin Haider Darwish']</t>
+          <t>['Areej Mohsin Haider Darwish', 'Areej Darwish', 'اريج محسن درويش', 'Areej Mohsin Darwish', 'Areej Mohsin Haider Darwish Al Zaabi']</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -1407,7 +1407,7 @@
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V6" t="n">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="AD6" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>['Amal Bahwan']</t>
+          <t>['Amal Bahwan', 'أمل بهوان']</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1577,7 +1577,7 @@
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V7" t="n">
@@ -1747,7 +1747,7 @@
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V8" t="n">
@@ -1778,12 +1778,12 @@
       </c>
       <c r="AD8" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>['Azza Al Ismaili']</t>
+          <t>['عزة الإسماعيلية', 'Азза Аль Ісмаїлі', 'Azza Al Ismaili', 'আজ্জা আল ইসমাইলি']</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1917,7 +1917,7 @@
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V9" t="n">
@@ -1948,12 +1948,12 @@
       </c>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>['Nashiah Al Kharousiyah', 'ناشئة بنت سعود الخروصية', "['Nashi'ah bint Saud Al Kharousiyah']", 'Nashiah Bint Saud Al Kharousiyah', 'Nashi Ah Bint Saud Bin Mohammed Al Kharousiyah']</t>
+          <t>['ناشئة بنت سعود الخروصية', "Nashi'ah bint Saud Al Kharousiyah", 'Nashiah Bint Saud Al Kharousiyah', 'Nashi Ah Bint Saud Bin Mohammed Al Kharousiyah', 'Nashiah Al Kharousiyah', 'ناشئة الخروصية']</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -2091,7 +2091,7 @@
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V10" t="n">
@@ -2122,12 +2122,12 @@
       </c>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>['Laila Bint Ahmed Bin Awad Al Najjar', 'Laila Bint Ahmed Bin Awadh Al Najar']</t>
+          <t>['Laila Bint Ahmed Bin Awadh Al Najar', 'Laila Binti Ahmed Ibn Avad Al Najjar', 'Laila Bint Ahmed Bin Awad Al Najjar', 'ليلى النجار']</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -2261,7 +2261,7 @@
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V11" t="n">
@@ -2431,7 +2431,7 @@
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V12" t="n">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>['Hind Bahwan', 'Sheikha Hind Bahwan', 'Hind S Bahwan']</t>
+          <t>['Hind S Bahwan', 'Hind Bahwan', 'Sheikha Hind Bahwan']</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -2601,7 +2601,7 @@
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V13" t="n">
@@ -2771,7 +2771,7 @@
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V14" t="n">
@@ -2802,12 +2802,12 @@
       </c>
       <c r="AD14" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>['Sayyida Rawan Ahmed Al Said', 'روان بنت أحمد بن ثابت آل سعيد', 'Rawan Ahmed Thabet Aal Saeed', 'Rawan Bint Ahmed Bin Thabit Al Said', 'Sayyidah Rawan Bint Ahmed Al Said', 'Rawan Al Said', 'Rawan Ahmed Thabit Al Said', 'Sayyeda Rawan Ahmed Al Said']</t>
+          <t>['Sayyeda Rawan Ahmed Al Said', 'روان آل سعيد', 'Rawan Al Said', 'روان بنت أحمد بن ثابت آل سعيد', 'Sayyidah Rawan Bint Ahmed Al Said', 'Rawan Bint Ahmed Bin Thabit Al Said', 'Rawan Ahmed Thabet Aal Saeed', 'Rawan Ahmed Thabit Al Said', 'Sayyida Rawan Ahmed Al Said']</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -2941,7 +2941,7 @@
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V15" t="n">
@@ -3111,7 +3111,7 @@
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V16" t="n">
@@ -3289,7 +3289,7 @@
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V17" t="n">
@@ -3320,12 +3320,12 @@
       </c>
       <c r="AD17" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE17" t="inlineStr">
         <is>
-          <t>['Arfah Bin Frijoon Bait Sameer', 'Arfah Bin Frijoon']</t>
+          <t>['Arfah Bin Frijoon Bait Sameer', 'عرفة بن فريجون', 'Arfah Bin Frijoon']</t>
         </is>
       </c>
       <c r="AF17" t="inlineStr">
@@ -3463,7 +3463,7 @@
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V18" t="n">
@@ -3494,12 +3494,12 @@
       </c>
       <c r="AD18" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE18" t="inlineStr">
         <is>
-          <t>['Rahma Bint Ibrahim Al Mahrouqi', 'Dr Rahma Bint Ibrahim Al Mahrooqi', 'Dr Rahma Bint Ibrahim Bin Said Al Mahrouqi', 'Rahma Bint Ibrahim Al Mahrooqi']</t>
+          <t>['Rahma Bint Ibrahim Al Mahrouqi', 'Rahma Bint Ibrahim Al Mahrooqi', 'Dr Rahma Bint Ibrahim Al Mahrooqi', 'رحمة المحروقي', 'রহমা বিনতে ইব্রাহিম আল মাহরুকি', 'Dr Rahma Bint Ibrahim Bin Said Al Mahrouqi']</t>
         </is>
       </c>
       <c r="AF18" t="inlineStr">
@@ -3637,7 +3637,7 @@
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V19" t="n">
@@ -3668,12 +3668,12 @@
       </c>
       <c r="AD19" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE19" t="inlineStr">
         <is>
-          <t>['Qais Mohammed Al Yousef', 'Qais Bin Mohammed Bin Moosa Al Yousef', 'Qais Al Yousef']</t>
+          <t>['Qais Mohammed Al Yousef', 'قيس محمد اليوسف', 'Qais Al Yousef', 'কায়েস মোহাম্মদ আল ইউসুফ', 'Qais Bin Mohammed Bin Moosa Al Yousef', 'Qays Muhammad Al Yusuf']</t>
         </is>
       </c>
       <c r="AF19" t="inlineStr">
@@ -3811,7 +3811,7 @@
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V20" t="n">
@@ -3842,12 +3842,12 @@
       </c>
       <c r="AD20" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE20" t="inlineStr">
         <is>
-          <t>['Salim Bin Nasir Bin Said Al Aufi', 'Salim Bin Nasser Al Aufi', 'Salem Al Oufi', 'Eng Salim Bin Nasir Bin Said Al Aufi']</t>
+          <t>['সালিম বিন নাসের বিন সাইদ আল আউফি', 'Eng Salim Bin Nasir Bin Said Al Aufi', 'سالم بن ناصر العوفي', 'Salim Bin Nasser Al Aufi', 'Salim Bin Nasir Bin Said Al Aufi', 'Salem Al Oufi', 'Salim Ibn Nosir Ibn Said Al Avfiy']</t>
         </is>
       </c>
       <c r="AF20" t="inlineStr">
@@ -3985,7 +3985,7 @@
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V21" t="n">
@@ -4016,12 +4016,12 @@
       </c>
       <c r="AD21" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE21" t="inlineStr">
         <is>
-          <t>['Salem Bin Mohammed Al Mahrouqi', 'Salim Bin Mohammed Bin Said Al Mahrouqi']</t>
+          <t>['Salim Ibn Muhammad Al Mahrukiy', 'Salim Bin Mohammed Bin Said Al Mahrouqi', 'سالم بن محمد المحروقي', 'Salem Bin Mohammed Al Mahrouqi', 'সালেম বিন মোহাম্মদ আল মাহরুকি']</t>
         </is>
       </c>
       <c r="AF21" t="inlineStr">
@@ -4155,7 +4155,7 @@
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V22" t="n">
@@ -4325,7 +4325,7 @@
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V23" t="n">
@@ -4361,7 +4361,7 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>['Nemah Al Busaidiyah', 'Nemah Bint Jamiel Bin Farhan Al Busaidiya']</t>
+          <t>['Nemah Bint Jamiel Bin Farhan Al Busaidiya', 'Nemah Al Busaidiyah']</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -4495,7 +4495,7 @@
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V24" t="n">
@@ -4665,7 +4665,7 @@
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V25" t="n">
@@ -4835,7 +4835,7 @@
       <c r="T26" t="inlineStr"/>
       <c r="U26" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V26" t="n">
@@ -5005,7 +5005,7 @@
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V27" t="n">
@@ -5179,7 +5179,7 @@
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V28" t="n">
@@ -5210,12 +5210,12 @@
       </c>
       <c r="AD28" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE28" t="inlineStr">
         <is>
-          <t>['Idris Bin Abdul Rahman Al Khanjari']</t>
+          <t>['إدريس بن عبد الرحمن الخنجري', 'Idris Bin Abdul Rahman Al Khanjari']</t>
         </is>
       </c>
       <c r="AF28" t="inlineStr">
@@ -5353,7 +5353,7 @@
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V29" t="n">
@@ -5384,12 +5384,12 @@
       </c>
       <c r="AD29" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Original Script Name']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE29" t="inlineStr">
         <is>
-          <t>['Khalid Al Mawali', 'Khalid Al Ma Awali', 'Khàlid al Maawalí']</t>
+          <t>['خالد المعولي', 'Khalid Al Mawali', 'Khalid Al Ma Awali', 'Khàlid al Maawalí']</t>
         </is>
       </c>
       <c r="AF29" t="inlineStr">
@@ -5535,7 +5535,7 @@
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V30" t="n">
@@ -5566,12 +5566,12 @@
       </c>
       <c r="AD30" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE30" t="inlineStr">
         <is>
-          <t>['Haitham Bin Tariq Al Said', 'Haitham Ibn Tariq', 'Hajtham bin Tárik Ál Saíd', 'Haitham Bin Tariq', "הית'ם בן טארק אאל סעיד", 'Sultan Haitham Bin Tariq Al Said', 'ハイサム・ビン・ターリク・アール＝サイード', 'Hàytham ibn Tàriq', 'Hajszam bin Tárik Ál Szaíd', 'Haitham Bin Tariq Bin Taymoar Al Said', 'Hajsám bin Tárik Saíd', 'Haitham bin Tariq al Busaíd', 'Heysem bin Tarık bin Teymur el Busaid', 'ہیثم بن طارق', 'السلطان هيثم بن طارق آل سعيد', 'Hàytham ibn Tàrq Al Saïd', 'Haïtham bin Tariq', 'Heysem bin Tarık bin Teymur el Said', 'Heysəm ibn Tariq']</t>
+          <t>['Ҳайсам ибни Ториқ Оли Саъид', 'Haitham bin Tariq al Busaíd', 'ハイサム・ビン・タリク・サイード', 'ハイサム・ビン・ターリク・アール＝サイード', 'ہیثم بن طارق آل سعید', 'ہیثم بن طارق', 'হাইসাম বিন তারিক আল সাইদ', 'Хайтам бин Тарик Ал Саид', 'Sultan Haitham Bin Tariq Al Said', 'Hàytham ibn Tàriq', 'Heysem bin Tarık bin Teymur el Said', 'Хайтем бен Тарік Аль Саїд', 'Haitham Bin Tarik Al Said', '하이탐 빈 타리크 알사이드', 'Haysam Ibn Toriq', '海赛姆·本·塔里克·阿勒赛义德', 'Χαϊθάμ μπιν Ταρίκ αλ Σαΐντ', "הית'ם בן טארק אאל סעיד", 'Хайтам Бін Тарык Аль Саід', 'Хајтем бин Тарик ел Саид', 'สมเด็จพระราชาธิบดีสุลต่านฮัยษัม บิน ฏอริก อาล ซะอีด', 'هیثم بن طارق', 'Хейсам бен Тарик Аль Саид', 'ھەیتەم کوڕی تارق ئال سەعید', 'Haitham de Omán', 'Һайсам бин Тарикъ Аль Саид', 'Heysem bin Tarık bin Teymur el Busaid', 'Haïtham ben Tariq', 'Hajtam Bin Tarik Al Sa Id', 'Haitham Bin Tariq Bin Taymoar Al Said', 'Hajtam Bin Tarik El Said', 'هيثم بن طارق آل سعيد', 'السلطان هيثم بن طارق آل سعيد', "היית'ם בן טארק אאל סעיד", 'Haitham Bin Tariq Al Said', 'Hajszam bin Tárik Ál Szaíd', 'Hajsám bin Tárik Saíd', 'Haitham ibn Ṭāriq Āl Saʿīd', 'Հայսամ բին Թարիք Ալ Սաիդ', 'हैथम बिन तारिक अल सईद', 'हैयथम बिन तारिक अल सइद', 'ஐத்தாம் பின் தாரிக் அல் சயீது', 'Haitham Tariqing', 'Хајтам Бин Тарик Ал Суад', 'ჰაითამ ბინ თარიქ ალ საიდი', 'Haitham Bin Tariq', 'Hàytham ibn Tàrq Al Saïd', 'Hajtham bin Tárik Ál Saíd', "Hajsam ibn Tarik Al Sa'id", 'Heysem bin Tarık El Said', 'هیثم بن طارق آل سعيد', 'Heysəm ibn Tariq', 'هيثم بن طارق', 'Haitham Ibn Tariq', 'Haïtham bin Tariq', 'Haytham Bin Tarik Al Sa Id', 'Hajszam ománi szultán', 'Haïtham bin Tariq Al Saïd', 'Haitham ibn Tāriq', 'Hajtham bin Tárik']</t>
         </is>
       </c>
       <c r="AF30" t="inlineStr">
@@ -5709,7 +5709,7 @@
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V31" t="n">
@@ -5879,7 +5879,7 @@
       <c r="T32" t="inlineStr"/>
       <c r="U32" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V32" t="n">
@@ -5915,7 +5915,7 @@
       </c>
       <c r="AE32" t="inlineStr">
         <is>
-          <t>['Maani Bint Abdullah Bin Hamad Al Busaidi', 'Sayyida Maani Bint Abdullah', 'Maani Al Busaidi']</t>
+          <t>['Maani Al Busaidi', 'Sayyida Maani Bint Abdullah', 'Maani Bint Abdullah Bin Hamad Al Busaidi']</t>
         </is>
       </c>
       <c r="AF32" t="inlineStr">
@@ -6049,7 +6049,7 @@
       <c r="T33" t="inlineStr"/>
       <c r="U33" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V33" t="n">
@@ -6219,7 +6219,7 @@
       <c r="T34" t="inlineStr"/>
       <c r="U34" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V34" t="n">
@@ -6250,12 +6250,12 @@
       </c>
       <c r="AD34" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE34" t="inlineStr">
         <is>
-          <t>['Samira Bint Mohamed Al Moosa']</t>
+          <t>['সামিরা বিনতে মোহাম্মদ আল মূসা', 'سميرة بنت محمد الموسى', 'סמירה בינת מוחמד אל מוסה', 'Samira Bint Mohamed Al Moosa']</t>
         </is>
       </c>
       <c r="AF34" t="inlineStr">
@@ -6397,7 +6397,7 @@
       <c r="T35" t="inlineStr"/>
       <c r="U35" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V35" t="n">
@@ -6428,12 +6428,12 @@
       </c>
       <c r="AD35" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE35" t="inlineStr">
         <is>
-          <t>['Munib El Masri', 'מוניב אל מסרי', 'Munib Rashid Al Masri', 'منيب المصري', 'Munib Al Masri', 'Mounib Al Masri', 'מניב אל מצרי', 'מניב אלמצרי']</t>
+          <t>['מוניב אל מסרי', 'Munib Rashid Al Masri', 'Munib Al Masri', 'Munib Masri', '穆尼布·马斯里', 'מניב אלמצרי', 'מניב אל מצרי', 'منيب المصري', 'Mounib Al Masri', 'Munib El Masri']</t>
         </is>
       </c>
       <c r="AF35" t="inlineStr">
@@ -6567,7 +6567,7 @@
       <c r="T36" t="inlineStr"/>
       <c r="U36" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V36" t="n">
@@ -6598,12 +6598,12 @@
       </c>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE36" t="inlineStr">
         <is>
-          <t>['Talal Sulaiman Al Rahbi', 'Talal Sulaiman Alrahbi', 'Talal Bin Suleiman Alrahbi']</t>
+          <t>['Talal Sulaiman Al Rahbi', 'طلال بن سليمان الرحبى', 'Talal Sulaiman Alrahbi', 'Talal Bin Suleiman Alrahbi']</t>
         </is>
       </c>
       <c r="AF36" t="inlineStr">
@@ -6741,7 +6741,7 @@
       <c r="T37" t="inlineStr"/>
       <c r="U37" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V37" t="n">
@@ -6772,12 +6772,12 @@
       </c>
       <c r="AD37" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE37" t="inlineStr">
         <is>
-          <t>['Salem Ben Nasser Ismaily', 'Salem Bin Nasser Al Ismaily', 'Salem Ben Nasser Al Ismaily']</t>
+          <t>['سالم بن ناصر الشنجل', 'Salem Nasser', 'Salem Ben Nasser Al Ismaily', 'সালিম বিন নাসের আল ইসমায়েলী', 'Salem Ben Nasser Ismaily', 'Salem Bin Nasser Al Ismaily']</t>
         </is>
       </c>
       <c r="AF37" t="inlineStr">
@@ -6911,7 +6911,7 @@
       <c r="T38" t="inlineStr"/>
       <c r="U38" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V38" t="n">
@@ -6942,12 +6942,12 @@
       </c>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE38" t="inlineStr">
         <is>
-          <t>['Aisha Bint Khalfan Bin Jameel']</t>
+          <t>['عائشة بنت خلفان بن جميل', 'Aisha Bint Khalfan Bin Jameel', 'আয়েশা বিনতে খালফান বিন জামিল']</t>
         </is>
       </c>
       <c r="AF38" t="inlineStr">
@@ -7085,7 +7085,7 @@
       <c r="T39" t="inlineStr"/>
       <c r="U39" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V39" t="n">
@@ -7116,12 +7116,12 @@
       </c>
       <c r="AD39" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE39" t="inlineStr">
         <is>
-          <t>['Dr Madeeha Bint Ahmed Bin Nassir Al Shibaniyah', 'Dr Madiha Bint Ahmad Bin Nasser Al Shibaniyah', 'Madeeha Bint Ahmed Bin Nassir Al Shibaniyah']</t>
+          <t>['Dr Madiha Bint Ahmad Bin Nasser Al Shibaniyah', 'Dr Madeeha Bint Ahmed Bin Nassir Al Shibaniyah', 'مديحة بنت أحمد بن ناصر الشيبانية', 'মাদেহা বিনতে আহমেদ বিন নাসির আল শিবানীয়া', 'Madeeha Bint Ahmed Bin Nassir Al Shibaniyah']</t>
         </is>
       </c>
       <c r="AF39" t="inlineStr">
@@ -7259,7 +7259,7 @@
       <c r="T40" t="inlineStr"/>
       <c r="U40" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V40" t="n">
@@ -7290,12 +7290,12 @@
       </c>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE40" t="inlineStr">
         <is>
-          <t>['Dr Abdullah Bin Muhammad Bin Said Al Saeedi', 'Abdullah Al Saidi']</t>
+          <t>['عبد الله بن محمد السعيدي', 'Abdullah Al Saidi', 'Dr Abdullah Bin Muhammad Bin Said Al Saeedi']</t>
         </is>
       </c>
       <c r="AF40" t="inlineStr">
@@ -7437,7 +7437,7 @@
       <c r="T41" t="inlineStr"/>
       <c r="U41" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V41" t="n">
@@ -7468,12 +7468,12 @@
       </c>
       <c r="AD41" t="inlineStr">
         <is>
-          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE41" t="inlineStr">
         <is>
-          <t>['يوسف بن علوي', 'ユーセフ・ビン・アラウィ・ビン・ アブダッラー・アル・イブラヒーム', "['Jusúf bin Alawi bin Abduláh']", 'Alawi Abdullah']</t>
+          <t>['Jusúf bin Alawi bin Abduláh', 'Youssef Bin Alawi Bin Abdullah', 'Alawi Abdullah', 'ユースフ・ビン・アラウィ・ビン・アブドゥッラー', '优素福·本·阿拉维·本·阿卜杜拉', 'Youssef Al Alawi Abdullah', 'ユーセフ・ビン・アラウィ・ビン・ アブダッラー・アル・イブラヒーム', 'يوسف بن علوي', 'Yusuf Bin Alawi Bin Abdullah', 'یوسف بن علوی', 'Юсуф бін Аляві бін Абдалла', 'ইউসুফ বিন আলাভি', 'يوسف بن علوى', 'יוסוף בן עלווי']</t>
         </is>
       </c>
       <c r="AF41" t="inlineStr">
@@ -7611,7 +7611,7 @@
       <c r="T42" t="inlineStr"/>
       <c r="U42" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V42" t="n">
@@ -7642,12 +7642,12 @@
       </c>
       <c r="AD42" t="inlineStr">
         <is>
-          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE42" t="inlineStr">
         <is>
-          <t>['السيد خالد', 'خالد بن حمد بن حمود', 'خالد بن حمد', 'السيد خالد بن حمد بن حمود البوسعيدي', 'Sayyid Khalid Bin Hilal Al Busaidi', 'السيد خالد البوسعيدي', 'Sayyid Khalid Bin Hilal Bin Saud Al Busaidi', 'السيد خالد بن حمد', 'خالد بن حمد بن حمود البوسعيدي', 'Khālid al Būsaʻīdī']</t>
+          <t>['خالد البوسعيدي', 'السيد خالد البوسعيدي', 'خالد بن حمد', 'Sayyid Khalid Bin Hilal Al Busaidi', 'السيد خالد بن حمد بن حمود البوسعيدي', 'Sayyid Khalid Bin Hilal Bin Saud Al Busaidi', 'السيد خالد', 'السيد خالد بن حمد', 'خالد بن حمد بن حمود البوسعيدي', 'خالد بن حمد بن حمود', 'خالد بن حمد آل خلیفه', 'Khālid al Būsaʻīdī']</t>
         </is>
       </c>
       <c r="AF42" t="inlineStr">
@@ -7793,7 +7793,7 @@
       <c r="T43" t="inlineStr"/>
       <c r="U43" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V43" t="n">
@@ -7824,12 +7824,12 @@
       </c>
       <c r="AD43" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE43" t="inlineStr">
         <is>
-          <t>['Asa Ad Bin Tariq', 'アスアド・ビン・ターリク・ビン・タイムール・アール・サイード', 'Asa Ad Bin Tariq Bin Taimur Al Said', 'アスアド・ビン・ターリク・アール・サイード', 'Asa Ad Al Said', 'Саїд Асад бен Тарік Аль Саїд', 'أسعد بن طارق بن تيمور آل سعيد', 'Asa Ad Bin Tariq Bin Taimur']</t>
+          <t>['アスアド・ビン・ターリク・アル＝サイード', 'Asa Ad Al Said', '阿萨德·本·塔里克', 'אסעד בן טארק', 'আসাদ বিন তারিক', 'Asa Ad Bin Tariq Bin Taimur', 'أسعد بن طارق بن تيمور آل سعيد', 'Asa Ad Bin Tariq', 'Асаад бен Тарік бен Таймур Аль Саїд', 'أسعد بن طارق', 'อาซาอัด บิน ฏอริก', 'Асад бин Тарик', 'Asa Ad Bin Tariq Bin Taimur Al Said', 'Assad Bin Tariq Al Said', 'アスアド・ビン・ターリク・ビン・タイムール・アール・サイード', 'アスアド・ビン・ターリク・アール・サイード', 'Саїд Асад бен Тарік Аль Саїд']</t>
         </is>
       </c>
       <c r="AF43" t="inlineStr">
@@ -7967,7 +7967,7 @@
       <c r="T44" t="inlineStr"/>
       <c r="U44" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V44" t="n">
@@ -7998,12 +7998,12 @@
       </c>
       <c r="AD44" t="inlineStr">
         <is>
-          <t>['Also Known As']</t>
+          <t>['Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE44" t="inlineStr">
         <is>
-          <t>['Khalid Bin Omar Bin Said Al Marhoon']</t>
+          <t>['خالد بن عمر المرهون', 'Khalid Bin Omar Bin Said Al Marhoon']</t>
         </is>
       </c>
       <c r="AF44" t="inlineStr">
@@ -8141,7 +8141,7 @@
       <c r="T45" t="inlineStr"/>
       <c r="U45" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V45" t="n">
@@ -8315,7 +8315,7 @@
       <c r="T46" t="inlineStr"/>
       <c r="U46" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V46" t="n">
@@ -8346,12 +8346,12 @@
       </c>
       <c r="AD46" t="inlineStr">
         <is>
-          <t>['Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE46" t="inlineStr">
         <is>
-          <t>['محمد بن حمد الرمحي', 'Mohammed Bin Hamad Al Rumhy', 'محمد بن حمد بن سيف الرمحي', 'H E Dr Mohammed Bin Hamad Al Rumhy', 'Muhammad Ibn Hamad Al Rumhi', 'Mohammed Al Rumhi']</t>
+          <t>['H E Dr Mohammed Bin Hamad Al Rumhy', 'Muhammad Ibn Hamad Al Rumhi', 'Mohammed Bin Hamad Al Rumhy', 'محمد بن حمد الرمحي', 'محمد بن حمد الرمحى', 'محمد بن حمد بن سيف الرمحي', 'Mohammed Al Rumhi']</t>
         </is>
       </c>
       <c r="AF46" t="inlineStr">
@@ -8485,7 +8485,7 @@
       <c r="T47" t="inlineStr"/>
       <c r="U47" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V47" t="n">
@@ -8516,12 +8516,12 @@
       </c>
       <c r="AD47" t="inlineStr">
         <is>
-          <t>['Original Script Name', 'Original Script Name', 'Also Known As']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE47" t="inlineStr">
         <is>
-          <t>['راوية البوسعيدية', "['Ravíja Saúd al Busaidi']", 'Rawya Bint Saud Al Busaidi']</t>
+          <t>['ראוויה סעוד אל בוסעידי', 'Ravíja Saúd al Busaidi', 'Rawya Bint Saud Al Busaidi', 'Rawya Saud Al Busaidi', 'راوية البوسعيدية']</t>
         </is>
       </c>
       <c r="AF47" t="inlineStr">
@@ -8663,7 +8663,7 @@
       <c r="T48" t="inlineStr"/>
       <c r="U48" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V48" t="n">
@@ -8694,12 +8694,12 @@
       </c>
       <c r="AD48" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE48" t="inlineStr">
         <is>
-          <t>['Shihab Bin Tariq Al Said', 'Hh Shihab Bin Tariq', 'Sultan Haitham Bin Tarik Al Said']</t>
+          <t>['شهاب بن طارق آل سعيد', 'شہاب بن طارق آل سعید', 'שיהאב בן טארק', 'Шихаб бен Тарік Аль Саїд', 'Шихаб бин Тарик', 'Shihab Bin Tariq Al Said', 'ชีฮับ บิน ฏอริก', 'শিহাব বিন তারিক', 'Sultan Haitham Bin Tarik Al Said', 'シハブ・ビン・ターリク・アール＝サイード', 'Hh Shihab Bin Tariq']</t>
         </is>
       </c>
       <c r="AF48" t="inlineStr">
@@ -8837,7 +8837,7 @@
       <c r="T49" t="inlineStr"/>
       <c r="U49" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V49" t="n">
@@ -8873,7 +8873,7 @@
       </c>
       <c r="AE49" t="inlineStr">
         <is>
-          <t>['عبد الله بن راشد السيابي', 'Abdullah Ibn Rashid Al Sayyabi', 'عبد الله بن راشد بن عزيز', 'عبد الله راشد عزيز السيابي', 'عبد الله  السيابي', 'عبد الله بن راشد بن عزيز السيابي', 'Abd Al Allah Ibn Rashid Ibn Aziz Al Sayyabi']</t>
+          <t>['عبد الله بن راشد بن عزيز السيابي', 'Abd Al Allah Ibn Rashid Ibn Aziz Al Sayyabi', 'عبد الله بن راشد بن عزيز', 'عبد الله راشد عزيز السيابي', 'عبد الله بن راشد السيابي', 'عبد الله  السيابي', 'Abdullah Ibn Rashid Al Sayyabi']</t>
         </is>
       </c>
       <c r="AF49" t="inlineStr">
@@ -9011,7 +9011,7 @@
       <c r="T50" t="inlineStr"/>
       <c r="U50" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V50" t="n">
@@ -9042,12 +9042,12 @@
       </c>
       <c r="AD50" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As']</t>
+          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Also Known As', 'Also Known As']</t>
         </is>
       </c>
       <c r="AE50" t="inlineStr">
         <is>
-          <t>['Hilal Bin Ali Bin Hilal Al Sabti', 'Dr Hilal Al Sabti', 'Hilal Al Sabti', 'Dr Hilal Bin Ali Bin Hilal Al Sabti', 'Hilal Bin Ali Al Sabti']</t>
+          <t>['Hilal Al Sabti', 'Hilal Bin Ali Al Sabti', 'Dr Hilal Al Sabti', 'هلال بن علي السبتي', 'Hilal Bin Ali Bin Hilal Al Sabti', 'Dr Hilal Bin Ali Bin Hilal Al Sabti']</t>
         </is>
       </c>
       <c r="AF50" t="inlineStr">
@@ -9189,7 +9189,7 @@
       <c r="T51" t="inlineStr"/>
       <c r="U51" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V51" t="n">
@@ -9220,12 +9220,12 @@
       </c>
       <c r="AD51" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name']</t>
+          <t>['Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE51" t="inlineStr">
         <is>
-          <t>['Amr Al Bidh', 'Amr Al Beidh', 'Бейд Амр', 'عمرو علي سالم البيض']</t>
+          <t>['Amr Al Beidh', 'Амр аль Бейд', 'عمرو البيض', 'Amr Al Bidh', 'Бейд Амр', 'عمرو علي سالم البيض']</t>
         </is>
       </c>
       <c r="AF51" t="inlineStr">
@@ -9367,7 +9367,7 @@
       <c r="T52" t="inlineStr"/>
       <c r="U52" t="inlineStr">
         <is>
-          <t>2025-12-27</t>
+          <t>2026-01-26</t>
         </is>
       </c>
       <c r="V52" t="n">
@@ -9398,12 +9398,12 @@
       </c>
       <c r="AD52" t="inlineStr">
         <is>
-          <t>['Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Original Script Name']</t>
+          <t>['Original Script Name', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Also Known As', 'Original Script Name', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name', 'Also Known As', 'Original Script Name']</t>
         </is>
       </c>
       <c r="AE52" t="inlineStr">
         <is>
-          <t>['Badr Al Busaidi', 'Sayyid Badr Bin Hamad Bin Hamood Al Busaidi', 'Sayyid Badr Albusaidi', 'Badr Bin Hamad Bin Hamood Al Busaidi', 'Sayyid Badr Bin Hamad Bin Hamoud Al Busaidi', 'サイイド・バドル・ビン・ハマド・ビン・ハムード・アルブーサイーディー', 'バドル・アル・ブサイディ', "['Badr bin Hamad el Búszajdi']"]</t>
+          <t>['サイイド・バドル・ビン・ハマド・ビン・ハムード・アルブーサイーディー', 'Sayyid Badr Bin Hamad Bin Hamoud Al Busaidi', 'バドル・アル・ブサイディ', '巴德尔·本·哈马德·本·哈姆德·布赛义迪', 'Sayyid Badr Bin Hamad Bin Hamood Al Busaidi', 'Sayyid Badr Albusaidi', 'بدر البوسعيدي', 'Badr bin Hamad el Búszajdi', 'Sayyid Badr Bin Hamad Bin Hamood Albusaidi', 'サイイド・バドア・ビン・ハマド・ビン・ハムード・アルブサイディ', 'Badr Bin Hamad Bin Hamood Al Busaidi', 'بدر البوسعیدی', 'Badr Al Busaidi', 'Бадр бін Хамад аль Бусаїді']</t>
         </is>
       </c>
       <c r="AF52" t="inlineStr">

</xml_diff>